<commit_message>
f1 added for req and arch
</commit_message>
<xml_diff>
--- a/outputs/evaluation/architecture/design/v1/CF_M01/CF_M01_arch_eval_avg.xlsx
+++ b/outputs/evaluation/architecture/design/v1/CF_M01/CF_M01_arch_eval_avg.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,6 +436,11 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>f1</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>mean semantic meaning</t>
         </is>
       </c>
@@ -452,7 +457,10 @@
       <c r="C2" t="n">
         <v>0.45</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="n">
+        <v>0.5881999999999999</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -471,6 +479,9 @@
         <v>0.5104</v>
       </c>
       <c r="D3" t="n">
+        <v>0.6351</v>
+      </c>
+      <c r="E3" t="n">
         <v>0.9832</v>
       </c>
     </row>
@@ -487,6 +498,9 @@
         <v>0.2083</v>
       </c>
       <c r="D4" t="n">
+        <v>0.3407</v>
+      </c>
+      <c r="E4" t="n">
         <v>0.8611</v>
       </c>
     </row>

</xml_diff>